<commit_message>
Caso 2 actualizado con datos reales del padron electoral de la ONPE
</commit_message>
<xml_diff>
--- a/caso2/resultado_miembros_mesa.xlsx
+++ b/caso2/resultado_miembros_mesa.xlsx
@@ -463,22 +463,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>NO ERES MIEMBRO DE MESA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CIUDADANO CONSULTADO</t>
+          <t>EDERD CARRASCO OSCCO</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AREQUIPA / AREQUIPA / JOSÉ LUIS BUSTAMANTE Y RIVERO</t>
+          <t>LIMA / LIMA / ATE</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>I.E. LOCAL DE VOTACIÓN ASIGNADO</t>
+          <t>IE 1244 MICAELA BASTIDAS - PROL AV LOS PORTALES DE PURUCHUCO</t>
         </is>
       </c>
     </row>

</xml_diff>